<commit_message>
Final polish: portable memory, approach slide, grader instructions
- Fix: the memory file stored absolute PDF paths, so a copied memory
  (e.g. the zip on another machine) made every known PDF unreadable.
  Known files are now re-pointed to where they are found; test added.
- Zip ships without the memory file so a grader's first run starts clean.
- Deck: new 'approach / how I split the time' slide (20 slides).
- README: tests need BEACON_DATA (they were silently skipped otherwise).
- Vendor readout: monthly totals carry cached values so previews show them.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6V2KMLCSVtUq6RnfYMNep
</commit_message>
<xml_diff>
--- a/Beacon Superday-Submission/output/Vendor_Readout.xlsx
+++ b/Beacon Superday-Submission/output/Vendor_Readout.xlsx
@@ -3443,31 +3443,31 @@
       </c>
       <c r="B11" s="5">
         <f>SUM(B2:B10)</f>
-        <v>0</v>
+        <v>23978261.68</v>
       </c>
       <c r="C11" s="5">
         <f>SUM(C2:C10)</f>
-        <v>0</v>
+        <v>1711799.87</v>
       </c>
       <c r="D11" s="5">
         <f>SUM(D2:D10)</f>
-        <v>0</v>
+        <v>107952.0</v>
       </c>
       <c r="E11" s="5">
         <f>SUM(E2:E10)</f>
-        <v>0</v>
+        <v>1508567.4</v>
       </c>
       <c r="F11" s="5">
         <f>SUM(F2:F10)</f>
-        <v>0</v>
+        <v>867316.8</v>
       </c>
       <c r="G11" s="5">
         <f>SUM(G2:G10)</f>
-        <v>0</v>
+        <v>13248.12</v>
       </c>
       <c r="H11" s="5">
         <f>SUM(H2:H10)</f>
-        <v>0</v>
+        <v>28187145.87</v>
       </c>
     </row>
     <row r="13" spans="1:10">

</xml_diff>